<commit_message>
feat(equipments): add category_raw filtering and UI
</commit_message>
<xml_diff>
--- a/dulieu.xlsx
+++ b/dulieu.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e69d5f0136af779a/Antigravity/quanly-ccdc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{ADDDC830-26A1-452B-BFA2-6861B21DDA51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{ADDDC830-26A1-452B-BFA2-6861B21DDA51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{730B3535-EF0E-4603-B278-70ED74695696}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{97EFADA0-FD0A-4F5A-861F-FD4F466C0038}"/>
   </bookViews>
@@ -19,7 +19,7 @@
     <externalReference r:id="rId2"/>
     <externalReference r:id="rId3"/>
   </externalReferences>
-  <calcPr calcId="191029" iterate="1"/>
+  <calcPr calcId="191029" iterate="1" calcCompleted="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -5092,7 +5092,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -5151,7 +5151,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -32037,7 +32036,7 @@
     <col min="25" max="25" width="2.140625" style="17" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" s="20" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
chore: remove stray files, keep scope to category-raw feature
</commit_message>
<xml_diff>
--- a/dulieu.xlsx
+++ b/dulieu.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e69d5f0136af779a/Antigravity/quanly-ccdc/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e69d5f0136af779a/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{ADDDC830-26A1-452B-BFA2-6861B21DDA51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{730B3535-EF0E-4603-B278-70ED74695696}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{ADDDC830-26A1-452B-BFA2-6861B21DDA51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4B24732C-D584-4A58-B5F0-4A9E56FB5B46}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{97EFADA0-FD0A-4F5A-861F-FD4F466C0038}"/>
   </bookViews>
@@ -19,7 +19,7 @@
     <externalReference r:id="rId2"/>
     <externalReference r:id="rId3"/>
   </externalReferences>
-  <calcPr calcId="191029" iterate="1" calcCompleted="0"/>
+  <calcPr calcId="191029" iterate="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>

</xml_diff>

<commit_message>
chore: fix stray files leaked into main, add .gitattributes for xlsx
</commit_message>
<xml_diff>
--- a/dulieu.xlsx
+++ b/dulieu.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e69d5f0136af779a/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e69d5f0136af779a/Antigravity/quanly-ccdc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{ADDDC830-26A1-452B-BFA2-6861B21DDA51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4B24732C-D584-4A58-B5F0-4A9E56FB5B46}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{ADDDC830-26A1-452B-BFA2-6861B21DDA51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{97EFADA0-FD0A-4F5A-861F-FD4F466C0038}"/>
   </bookViews>
@@ -5092,7 +5092,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -5151,6 +5151,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -32036,7 +32037,7 @@
     <col min="25" max="25" width="2.140625" style="17" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25" s="20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>

</xml_diff>